<commit_message>
Implement model selection with `--select` flag, enforce YAML and source file validation, update CLI, and refine engine logic
</commit_message>
<xml_diff>
--- a/output/enriched_orders.xlsx
+++ b/output/enriched_orders.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,28 +434,18 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>total</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>total</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
           <t>email</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>tier</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -464,31 +454,21 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>North</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>150</v>
-      </c>
-      <c r="F2" t="inlineStr">
+          <t>East</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>275.5</v>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>alice@example.com</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>gold</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -497,31 +477,21 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>North</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>75.5</v>
-      </c>
-      <c r="F3" t="inlineStr">
+          <t>South</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>180</v>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>charlie@example.com</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>bronze</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -530,101 +500,71 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>East</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>320</v>
-      </c>
-      <c r="F4" t="inlineStr">
+          <t>North</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>65</v>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>diana@example.com</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>gold</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Alice</t>
+          <t>Eve</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>South</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>95</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>alice@example.com</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>gold</t>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>88</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>eve@example.com</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Eve</t>
+          <t>Frank</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>East</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>65</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>eve@example.com</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>silver</t>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>440</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>frank@example.com</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Charlie</t>
+          <t>Alice</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -632,61 +572,41 @@
           <t>South</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>180</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>charlie@example.com</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>bronze</t>
+      <c r="D7" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>alice@example.com</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alice</t>
+          <t>Charlie</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>East</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>275.5</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>alice@example.com</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>gold</t>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>75.5</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>charlie@example.com</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -695,68 +615,48 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>North</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>65</v>
-      </c>
-      <c r="F9" t="inlineStr">
+          <t>East</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>320</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>diana@example.com</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>gold</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Frank</t>
+          <t>Eve</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>West</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>440</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>frank@example.com</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>bronze</t>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>65</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>eve@example.com</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Eve</t>
+          <t>Alice</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -764,22 +664,12 @@
           <t>North</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>88</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>eve@example.com</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>silver</t>
+      <c r="D11" t="n">
+        <v>150</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>alice@example.com</t>
         </is>
       </c>
     </row>

</xml_diff>